<commit_message>
More models per ticker (pre tp generation)
</commit_message>
<xml_diff>
--- a/order_df_export.xlsx
+++ b/order_df_export.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="150">
   <si>
     <t>ID</t>
   </si>
@@ -290,6 +290,117 @@
   </si>
   <si>
     <t>16906397265788548</t>
+  </si>
+  <si>
+    <t>16907022819464166</t>
+  </si>
+  <si>
+    <t>16907024471818676</t>
+  </si>
+  <si>
+    <t>16907030461335301</t>
+  </si>
+  <si>
+    <t>1690703059028976</t>
+  </si>
+  <si>
+    <t>16907037973001246</t>
+  </si>
+  <si>
+    <t>16907037973658526</t>
+  </si>
+  <si>
+    <t>1690703803832576</t>
+  </si>
+  <si>
+    <t>16907042625756557</t>
+  </si>
+  <si>
+    <t>16907042695043964</t>
+  </si>
+  <si>
+    <t>16907042701988053</t>
+  </si>
+  <si>
+    <t>1690704270334266</t>
+  </si>
+  <si>
+    <t>1690704276887927</t>
+  </si>
+  <si>
+    <t>1690704276974473</t>
+  </si>
+  <si>
+    <t>16907042773807168</t>
+  </si>
+  <si>
+    <t>16907042838338497</t>
+  </si>
+  <si>
+    <t>16907042842463574</t>
+  </si>
+  <si>
+    <t>16907042844683566</t>
+  </si>
+  <si>
+    <t>1690704291045862</t>
+  </si>
+  <si>
+    <t>16907042911594636</t>
+  </si>
+  <si>
+    <t>16907042913810885</t>
+  </si>
+  <si>
+    <t>16907042916141741</t>
+  </si>
+  <si>
+    <t>1690704297927563</t>
+  </si>
+  <si>
+    <t>1690704298020009</t>
+  </si>
+  <si>
+    <t>1690704298373023</t>
+  </si>
+  <si>
+    <t>16907042985326838</t>
+  </si>
+  <si>
+    <t>16907043050781229</t>
+  </si>
+  <si>
+    <t>1690704305167457</t>
+  </si>
+  <si>
+    <t>16907043053561075</t>
+  </si>
+  <si>
+    <t>16907043057449539</t>
+  </si>
+  <si>
+    <t>16907043121817968</t>
+  </si>
+  <si>
+    <t>1690704312274777</t>
+  </si>
+  <si>
+    <t>16907043125937507</t>
+  </si>
+  <si>
+    <t>16907043127219996</t>
+  </si>
+  <si>
+    <t>16907043191089003</t>
+  </si>
+  <si>
+    <t>16907043192118406</t>
+  </si>
+  <si>
+    <t>16907043194188266</t>
+  </si>
+  <si>
+    <t>16907043195456698</t>
   </si>
   <si>
     <t>EURUSD;rhi888806</t>
@@ -714,7 +825,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q77"/>
+  <dimension ref="A1:Q114"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:17">
@@ -778,16 +889,16 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>92</v>
+        <v>129</v>
       </c>
       <c r="E2" s="2">
         <v>45136.59542466338</v>
       </c>
       <c r="P2" t="s">
-        <v>106</v>
+        <v>143</v>
       </c>
       <c r="Q2" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -801,16 +912,16 @@
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E3" s="2">
         <v>45136.59720025676</v>
       </c>
       <c r="P3" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q3" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -824,16 +935,16 @@
         <v>1</v>
       </c>
       <c r="D4" t="s">
-        <v>94</v>
+        <v>131</v>
       </c>
       <c r="E4" s="2">
         <v>45136.60363814366</v>
       </c>
       <c r="P4" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q4" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="5" spans="1:17">
@@ -847,16 +958,16 @@
         <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>94</v>
+        <v>131</v>
       </c>
       <c r="E5" s="2">
         <v>45136.60377729374</v>
       </c>
       <c r="P5" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q5" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="6" spans="1:17">
@@ -870,16 +981,16 @@
         <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>92</v>
+        <v>129</v>
       </c>
       <c r="E6" s="2">
         <v>45136.64437173348</v>
       </c>
       <c r="P6" t="s">
-        <v>106</v>
+        <v>143</v>
       </c>
       <c r="Q6" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="7" spans="1:17">
@@ -893,16 +1004,16 @@
         <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E7" s="2">
         <v>45136.64611581015</v>
       </c>
       <c r="P7" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q7" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="8" spans="1:17">
@@ -916,16 +1027,16 @@
         <v>1</v>
       </c>
       <c r="D8" t="s">
-        <v>94</v>
+        <v>131</v>
       </c>
       <c r="E8" s="2">
         <v>45136.65247193063</v>
       </c>
       <c r="P8" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q8" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -939,16 +1050,16 @@
         <v>1</v>
       </c>
       <c r="D9" t="s">
-        <v>94</v>
+        <v>131</v>
       </c>
       <c r="E9" s="2">
         <v>45136.65260950934</v>
       </c>
       <c r="P9" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q9" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="10" spans="1:17">
@@ -962,16 +1073,16 @@
         <v>1</v>
       </c>
       <c r="D10" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E10" s="2">
         <v>45136.66043727005</v>
       </c>
       <c r="P10" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q10" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -985,16 +1096,16 @@
         <v>1</v>
       </c>
       <c r="D11" t="s">
-        <v>95</v>
+        <v>132</v>
       </c>
       <c r="E11" s="2">
         <v>45136.66043740383</v>
       </c>
       <c r="P11" t="s">
-        <v>108</v>
+        <v>145</v>
       </c>
       <c r="Q11" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -1008,16 +1119,16 @@
         <v>1</v>
       </c>
       <c r="D12" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E12" s="2">
         <v>45136.66050841245</v>
       </c>
       <c r="P12" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q12" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="13" spans="1:17">
@@ -1031,16 +1142,16 @@
         <v>1</v>
       </c>
       <c r="D13" t="s">
-        <v>92</v>
+        <v>129</v>
       </c>
       <c r="E13" s="2">
         <v>45136.66536320822</v>
       </c>
       <c r="P13" t="s">
-        <v>106</v>
+        <v>143</v>
       </c>
       <c r="Q13" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="14" spans="1:17">
@@ -1054,16 +1165,16 @@
         <v>1</v>
       </c>
       <c r="D14" t="s">
-        <v>92</v>
+        <v>129</v>
       </c>
       <c r="E14" s="2">
         <v>45136.66543679257</v>
       </c>
       <c r="P14" t="s">
-        <v>106</v>
+        <v>143</v>
       </c>
       <c r="Q14" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="15" spans="1:17">
@@ -1077,16 +1188,16 @@
         <v>1</v>
       </c>
       <c r="D15" t="s">
-        <v>95</v>
+        <v>132</v>
       </c>
       <c r="E15" s="2">
         <v>45136.66543702583</v>
       </c>
       <c r="P15" t="s">
-        <v>108</v>
+        <v>145</v>
       </c>
       <c r="Q15" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="16" spans="1:17">
@@ -1100,19 +1211,19 @@
         <v>1</v>
       </c>
       <c r="D16" t="s">
-        <v>96</v>
+        <v>133</v>
       </c>
       <c r="E16" s="2">
         <v>45136.66543719729</v>
       </c>
       <c r="O16" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P16" t="s">
-        <v>109</v>
+        <v>146</v>
       </c>
       <c r="Q16" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="17" spans="1:17">
@@ -1126,16 +1237,16 @@
         <v>1</v>
       </c>
       <c r="D17" t="s">
-        <v>92</v>
+        <v>129</v>
       </c>
       <c r="E17" s="2">
         <v>45136.66551153561</v>
       </c>
       <c r="P17" t="s">
-        <v>106</v>
+        <v>143</v>
       </c>
       <c r="Q17" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="18" spans="1:17">
@@ -1149,19 +1260,19 @@
         <v>1</v>
       </c>
       <c r="D18" t="s">
-        <v>97</v>
+        <v>134</v>
       </c>
       <c r="E18" s="2">
         <v>45136.66551169882</v>
       </c>
       <c r="O18" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P18" t="s">
-        <v>110</v>
+        <v>147</v>
       </c>
       <c r="Q18" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="19" spans="1:17">
@@ -1175,19 +1286,19 @@
         <v>1</v>
       </c>
       <c r="D19" t="s">
-        <v>96</v>
+        <v>133</v>
       </c>
       <c r="E19" s="2">
         <v>45136.6655122118</v>
       </c>
       <c r="O19" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P19" t="s">
-        <v>109</v>
+        <v>146</v>
       </c>
       <c r="Q19" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="20" spans="1:17">
@@ -1201,16 +1312,16 @@
         <v>1</v>
       </c>
       <c r="D20" t="s">
-        <v>92</v>
+        <v>129</v>
       </c>
       <c r="E20" s="2">
         <v>45136.66558442353</v>
       </c>
       <c r="P20" t="s">
-        <v>106</v>
+        <v>143</v>
       </c>
       <c r="Q20" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="21" spans="1:17">
@@ -1224,19 +1335,19 @@
         <v>1</v>
       </c>
       <c r="D21" t="s">
-        <v>96</v>
+        <v>133</v>
       </c>
       <c r="E21" s="2">
         <v>45136.66558458201</v>
       </c>
       <c r="O21" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P21" t="s">
-        <v>109</v>
+        <v>146</v>
       </c>
       <c r="Q21" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="22" spans="1:17">
@@ -1250,16 +1361,16 @@
         <v>1</v>
       </c>
       <c r="D22" t="s">
-        <v>92</v>
+        <v>129</v>
       </c>
       <c r="E22" s="2">
         <v>45136.6656575117</v>
       </c>
       <c r="P22" t="s">
-        <v>106</v>
+        <v>143</v>
       </c>
       <c r="Q22" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="23" spans="1:17">
@@ -1273,16 +1384,16 @@
         <v>1</v>
       </c>
       <c r="D23" t="s">
-        <v>97</v>
+        <v>134</v>
       </c>
       <c r="E23" s="2">
         <v>45136.66565766856</v>
       </c>
       <c r="P23" t="s">
-        <v>110</v>
+        <v>147</v>
       </c>
       <c r="Q23" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="24" spans="1:17">
@@ -1296,19 +1407,19 @@
         <v>1</v>
       </c>
       <c r="D24" t="s">
-        <v>95</v>
+        <v>132</v>
       </c>
       <c r="E24" s="2">
         <v>45136.66565783114</v>
       </c>
       <c r="O24" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P24" t="s">
-        <v>108</v>
+        <v>145</v>
       </c>
       <c r="Q24" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="25" spans="1:17">
@@ -1322,16 +1433,16 @@
         <v>1</v>
       </c>
       <c r="D25" t="s">
-        <v>98</v>
+        <v>135</v>
       </c>
       <c r="E25" s="2">
         <v>45136.66565799346</v>
       </c>
       <c r="P25" t="s">
-        <v>109</v>
+        <v>146</v>
       </c>
       <c r="Q25" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="26" spans="1:17">
@@ -1345,16 +1456,16 @@
         <v>1</v>
       </c>
       <c r="D26" t="s">
-        <v>92</v>
+        <v>129</v>
       </c>
       <c r="E26" s="2">
         <v>45136.66573147161</v>
       </c>
       <c r="P26" t="s">
-        <v>106</v>
+        <v>143</v>
       </c>
       <c r="Q26" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="27" spans="1:17">
@@ -1368,19 +1479,19 @@
         <v>1</v>
       </c>
       <c r="D27" t="s">
-        <v>97</v>
+        <v>134</v>
       </c>
       <c r="E27" s="2">
         <v>45136.66573165503</v>
       </c>
       <c r="O27" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P27" t="s">
-        <v>110</v>
+        <v>147</v>
       </c>
       <c r="Q27" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="28" spans="1:17">
@@ -1394,19 +1505,19 @@
         <v>1</v>
       </c>
       <c r="D28" t="s">
-        <v>95</v>
+        <v>132</v>
       </c>
       <c r="E28" s="2">
         <v>45136.66573181393</v>
       </c>
       <c r="O28" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P28" t="s">
-        <v>108</v>
+        <v>145</v>
       </c>
       <c r="Q28" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="29" spans="1:17">
@@ -1420,19 +1531,19 @@
         <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>96</v>
+        <v>133</v>
       </c>
       <c r="E29" s="2">
         <v>45136.66573217484</v>
       </c>
       <c r="O29" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P29" t="s">
-        <v>109</v>
+        <v>146</v>
       </c>
       <c r="Q29" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="30" spans="1:17">
@@ -1446,16 +1557,16 @@
         <v>1</v>
       </c>
       <c r="D30" t="s">
-        <v>92</v>
+        <v>129</v>
       </c>
       <c r="E30" s="2">
         <v>45136.66580540832</v>
       </c>
       <c r="P30" t="s">
-        <v>106</v>
+        <v>143</v>
       </c>
       <c r="Q30" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="31" spans="1:17">
@@ -1469,16 +1580,16 @@
         <v>1</v>
       </c>
       <c r="D31" t="s">
-        <v>99</v>
+        <v>136</v>
       </c>
       <c r="E31" s="2">
         <v>45136.66580557234</v>
       </c>
       <c r="P31" t="s">
-        <v>110</v>
+        <v>147</v>
       </c>
       <c r="Q31" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="32" spans="1:17">
@@ -1492,19 +1603,19 @@
         <v>1</v>
       </c>
       <c r="D32" t="s">
-        <v>100</v>
+        <v>137</v>
       </c>
       <c r="E32" s="2">
         <v>45136.66580572949</v>
       </c>
       <c r="O32" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P32" t="s">
-        <v>108</v>
+        <v>145</v>
       </c>
       <c r="Q32" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="33" spans="1:17">
@@ -1518,19 +1629,19 @@
         <v>1</v>
       </c>
       <c r="D33" t="s">
-        <v>96</v>
+        <v>133</v>
       </c>
       <c r="E33" s="2">
         <v>45136.66580684966</v>
       </c>
       <c r="O33" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P33" t="s">
-        <v>109</v>
+        <v>146</v>
       </c>
       <c r="Q33" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="34" spans="1:17">
@@ -1544,16 +1655,16 @@
         <v>1</v>
       </c>
       <c r="D34" t="s">
-        <v>92</v>
+        <v>129</v>
       </c>
       <c r="E34" s="2">
         <v>45136.66588032414</v>
       </c>
       <c r="P34" t="s">
-        <v>106</v>
+        <v>143</v>
       </c>
       <c r="Q34" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="35" spans="1:17">
@@ -1567,16 +1678,16 @@
         <v>1</v>
       </c>
       <c r="D35" t="s">
-        <v>97</v>
+        <v>134</v>
       </c>
       <c r="E35" s="2">
         <v>45136.6658804825</v>
       </c>
       <c r="P35" t="s">
-        <v>110</v>
+        <v>147</v>
       </c>
       <c r="Q35" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="36" spans="1:17">
@@ -1590,19 +1701,19 @@
         <v>1</v>
       </c>
       <c r="D36" t="s">
-        <v>100</v>
+        <v>137</v>
       </c>
       <c r="E36" s="2">
         <v>45136.66588066255</v>
       </c>
       <c r="O36" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P36" t="s">
-        <v>108</v>
+        <v>145</v>
       </c>
       <c r="Q36" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="37" spans="1:17">
@@ -1616,19 +1727,19 @@
         <v>1</v>
       </c>
       <c r="D37" t="s">
-        <v>96</v>
+        <v>133</v>
       </c>
       <c r="E37" s="2">
         <v>45136.66588111146</v>
       </c>
       <c r="O37" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P37" t="s">
-        <v>109</v>
+        <v>146</v>
       </c>
       <c r="Q37" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="38" spans="1:17">
@@ -1642,16 +1753,16 @@
         <v>1</v>
       </c>
       <c r="D38" t="s">
-        <v>92</v>
+        <v>129</v>
       </c>
       <c r="E38" s="2">
         <v>45136.66595374174</v>
       </c>
       <c r="P38" t="s">
-        <v>106</v>
+        <v>143</v>
       </c>
       <c r="Q38" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="39" spans="1:17">
@@ -1665,16 +1776,16 @@
         <v>1</v>
       </c>
       <c r="D39" t="s">
-        <v>99</v>
+        <v>136</v>
       </c>
       <c r="E39" s="2">
         <v>45136.66595390173</v>
       </c>
       <c r="P39" t="s">
-        <v>110</v>
+        <v>147</v>
       </c>
       <c r="Q39" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="40" spans="1:17">
@@ -1688,16 +1799,16 @@
         <v>1</v>
       </c>
       <c r="D40" t="s">
-        <v>101</v>
+        <v>138</v>
       </c>
       <c r="E40" s="2">
         <v>45136.66595405956</v>
       </c>
       <c r="P40" t="s">
-        <v>108</v>
+        <v>145</v>
       </c>
       <c r="Q40" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="41" spans="1:17">
@@ -1711,16 +1822,16 @@
         <v>1</v>
       </c>
       <c r="D41" t="s">
-        <v>98</v>
+        <v>135</v>
       </c>
       <c r="E41" s="2">
         <v>45136.66595424808</v>
       </c>
       <c r="P41" t="s">
-        <v>109</v>
+        <v>146</v>
       </c>
       <c r="Q41" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="42" spans="1:17">
@@ -1734,19 +1845,19 @@
         <v>1</v>
       </c>
       <c r="D42" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E42" s="2">
         <v>45136.6667292386</v>
       </c>
       <c r="O42" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P42" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q42" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="43" spans="1:17">
@@ -1760,19 +1871,19 @@
         <v>1</v>
       </c>
       <c r="D43" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E43" s="2">
         <v>45136.66687173695</v>
       </c>
       <c r="O43" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P43" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q43" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="44" spans="1:17">
@@ -1786,16 +1897,16 @@
         <v>1</v>
       </c>
       <c r="D44" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E44" s="2">
         <v>45136.66694286956</v>
       </c>
       <c r="P44" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q44" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="45" spans="1:17">
@@ -1809,16 +1920,16 @@
         <v>1</v>
       </c>
       <c r="D45" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E45" s="2">
         <v>45136.66812766632</v>
       </c>
       <c r="P45" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q45" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="46" spans="1:17">
@@ -1832,19 +1943,19 @@
         <v>1</v>
       </c>
       <c r="D46" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E46" s="2">
         <v>45136.66966999102</v>
       </c>
       <c r="O46" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P46" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q46" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="47" spans="1:17">
@@ -1858,19 +1969,19 @@
         <v>1</v>
       </c>
       <c r="D47" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E47" s="2">
         <v>45136.6697415712</v>
       </c>
       <c r="O47" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P47" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q47" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="48" spans="1:17">
@@ -1884,19 +1995,19 @@
         <v>1</v>
       </c>
       <c r="D48" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E48" s="2">
         <v>45136.66988432121</v>
       </c>
       <c r="O48" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P48" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q48" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="49" spans="1:17">
@@ -1910,19 +2021,19 @@
         <v>1</v>
       </c>
       <c r="D49" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E49" s="2">
         <v>45136.66995682847</v>
       </c>
       <c r="O49" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P49" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q49" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="50" spans="1:17">
@@ -1936,19 +2047,19 @@
         <v>1</v>
       </c>
       <c r="D50" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E50" s="2">
         <v>45136.67002962553</v>
       </c>
       <c r="O50" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P50" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q50" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="51" spans="1:17">
@@ -1962,19 +2073,19 @@
         <v>1</v>
       </c>
       <c r="D51" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E51" s="2">
         <v>45136.67010194205</v>
       </c>
       <c r="O51" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P51" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q51" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="52" spans="1:17">
@@ -1988,19 +2099,19 @@
         <v>1</v>
       </c>
       <c r="D52" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E52" s="2">
         <v>45136.67017347417</v>
       </c>
       <c r="O52" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P52" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q52" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="53" spans="1:17">
@@ -2014,19 +2125,19 @@
         <v>1</v>
       </c>
       <c r="D53" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E53" s="2">
         <v>45136.67024591174</v>
       </c>
       <c r="O53" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P53" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q53" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="54" spans="1:17">
@@ -2040,19 +2151,19 @@
         <v>1</v>
       </c>
       <c r="D54" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E54" s="2">
         <v>45136.67031751607</v>
       </c>
       <c r="O54" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P54" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q54" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="55" spans="1:17">
@@ -2066,19 +2177,19 @@
         <v>1</v>
       </c>
       <c r="D55" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E55" s="2">
         <v>45136.67046134384</v>
       </c>
       <c r="O55" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P55" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q55" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="56" spans="1:17">
@@ -2092,19 +2203,19 @@
         <v>1</v>
       </c>
       <c r="D56" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E56" s="2">
         <v>45136.67053319368</v>
       </c>
       <c r="O56" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P56" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q56" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="57" spans="1:17">
@@ -2118,19 +2229,19 @@
         <v>1</v>
       </c>
       <c r="D57" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E57" s="2">
         <v>45136.67060639364</v>
       </c>
       <c r="O57" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P57" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q57" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="58" spans="1:17">
@@ -2144,16 +2255,16 @@
         <v>1</v>
       </c>
       <c r="D58" t="s">
-        <v>92</v>
+        <v>129</v>
       </c>
       <c r="E58" s="2">
         <v>45136.67067973952</v>
       </c>
       <c r="P58" t="s">
-        <v>106</v>
+        <v>143</v>
       </c>
       <c r="Q58" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="59" spans="1:17">
@@ -2167,19 +2278,19 @@
         <v>1</v>
       </c>
       <c r="D59" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E59" s="2">
         <v>45136.67067991087</v>
       </c>
       <c r="O59" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P59" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q59" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="60" spans="1:17">
@@ -2193,16 +2304,16 @@
         <v>1</v>
       </c>
       <c r="D60" t="s">
-        <v>92</v>
+        <v>129</v>
       </c>
       <c r="E60" s="2">
         <v>45136.67075289096</v>
       </c>
       <c r="P60" t="s">
-        <v>106</v>
+        <v>143</v>
       </c>
       <c r="Q60" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="61" spans="1:17">
@@ -2216,19 +2327,19 @@
         <v>1</v>
       </c>
       <c r="D61" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E61" s="2">
         <v>45136.67075307867</v>
       </c>
       <c r="O61" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P61" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q61" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="62" spans="1:17">
@@ -2242,19 +2353,19 @@
         <v>1</v>
       </c>
       <c r="D62" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E62" s="2">
         <v>45136.67082601101</v>
       </c>
       <c r="O62" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P62" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q62" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="63" spans="1:17">
@@ -2268,16 +2379,16 @@
         <v>1</v>
       </c>
       <c r="D63" t="s">
-        <v>94</v>
+        <v>131</v>
       </c>
       <c r="E63" s="2">
         <v>45136.6708978409</v>
       </c>
       <c r="P63" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q63" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="64" spans="1:17">
@@ -2291,19 +2402,19 @@
         <v>1</v>
       </c>
       <c r="D64" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E64" s="2">
         <v>45136.67097071325</v>
       </c>
       <c r="O64" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P64" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q64" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="65" spans="1:17">
@@ -2317,16 +2428,16 @@
         <v>1</v>
       </c>
       <c r="D65" t="s">
-        <v>94</v>
+        <v>131</v>
       </c>
       <c r="E65" s="2">
         <v>45136.67104186679</v>
       </c>
       <c r="P65" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q65" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="66" spans="1:17">
@@ -2340,19 +2451,19 @@
         <v>1</v>
       </c>
       <c r="D66" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E66" s="2">
         <v>45136.67111350768</v>
       </c>
       <c r="O66" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P66" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q66" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="67" spans="1:17">
@@ -2366,16 +2477,16 @@
         <v>1</v>
       </c>
       <c r="D67" t="s">
-        <v>94</v>
+        <v>131</v>
       </c>
       <c r="E67" s="2">
         <v>45136.67139773812</v>
       </c>
       <c r="P67" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q67" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="68" spans="1:17">
@@ -2389,16 +2500,16 @@
         <v>1</v>
       </c>
       <c r="D68" t="s">
-        <v>94</v>
+        <v>131</v>
       </c>
       <c r="E68" s="2">
         <v>45136.67168082331</v>
       </c>
       <c r="P68" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q68" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="69" spans="1:17">
@@ -2412,19 +2523,19 @@
         <v>1</v>
       </c>
       <c r="D69" t="s">
-        <v>102</v>
+        <v>139</v>
       </c>
       <c r="E69" s="2">
         <v>45136.67217979555</v>
       </c>
       <c r="O69" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P69" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q69" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="70" spans="1:17">
@@ -2438,19 +2549,19 @@
         <v>1</v>
       </c>
       <c r="D70" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E70" s="2">
         <v>45136.67225350921</v>
       </c>
       <c r="O70" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P70" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q70" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="71" spans="1:17">
@@ -2464,19 +2575,19 @@
         <v>1</v>
       </c>
       <c r="D71" t="s">
-        <v>102</v>
+        <v>139</v>
       </c>
       <c r="E71" s="2">
         <v>45136.67232685709</v>
       </c>
       <c r="O71" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P71" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q71" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="72" spans="1:17">
@@ -2490,19 +2601,19 @@
         <v>1</v>
       </c>
       <c r="D72" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E72" s="2">
         <v>45136.67239956577</v>
       </c>
       <c r="O72" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P72" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q72" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="73" spans="1:17">
@@ -2516,19 +2627,19 @@
         <v>1</v>
       </c>
       <c r="D73" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E73" s="2">
         <v>45136.6724732099</v>
       </c>
       <c r="O73" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P73" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q73" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="74" spans="1:17">
@@ -2542,19 +2653,19 @@
         <v>1</v>
       </c>
       <c r="D74" t="s">
-        <v>102</v>
+        <v>139</v>
       </c>
       <c r="E74" s="2">
         <v>45136.67254701501</v>
       </c>
       <c r="O74" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P74" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q74" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="75" spans="1:17">
@@ -2568,16 +2679,16 @@
         <v>1</v>
       </c>
       <c r="D75" t="s">
-        <v>103</v>
+        <v>140</v>
       </c>
       <c r="E75" s="2">
         <v>45136.67269280797</v>
       </c>
       <c r="P75" t="s">
-        <v>110</v>
+        <v>147</v>
       </c>
       <c r="Q75" t="s">
-        <v>112</v>
+        <v>149</v>
       </c>
     </row>
     <row r="76" spans="1:17">
@@ -2591,19 +2702,19 @@
         <v>1</v>
       </c>
       <c r="D76" t="s">
-        <v>93</v>
+        <v>130</v>
       </c>
       <c r="E76" s="2">
         <v>45136.67269302224</v>
       </c>
       <c r="O76" t="s">
-        <v>105</v>
+        <v>142</v>
       </c>
       <c r="P76" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="Q76" t="s">
-        <v>111</v>
+        <v>148</v>
       </c>
     </row>
     <row r="77" spans="1:17">
@@ -2617,16 +2728,903 @@
         <v>1</v>
       </c>
       <c r="D77" t="s">
-        <v>104</v>
+        <v>141</v>
       </c>
       <c r="E77" s="2">
         <v>45136.67276579243</v>
       </c>
       <c r="P77" t="s">
+        <v>144</v>
+      </c>
+      <c r="Q77" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="78" spans="1:17">
+      <c r="A78" s="1">
+        <v>76</v>
+      </c>
+      <c r="B78" t="s">
+        <v>92</v>
+      </c>
+      <c r="C78">
+        <v>1</v>
+      </c>
+      <c r="D78" t="s">
+        <v>129</v>
+      </c>
+      <c r="E78" s="2">
+        <v>45137.39678576983</v>
+      </c>
+      <c r="P78" t="s">
+        <v>143</v>
+      </c>
+      <c r="Q78" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="79" spans="1:17">
+      <c r="A79" s="1">
+        <v>77</v>
+      </c>
+      <c r="B79" t="s">
+        <v>93</v>
+      </c>
+      <c r="C79">
+        <v>1</v>
+      </c>
+      <c r="D79" t="s">
+        <v>130</v>
+      </c>
+      <c r="E79" s="2">
+        <v>45137.39869549485</v>
+      </c>
+      <c r="P79" t="s">
+        <v>144</v>
+      </c>
+      <c r="Q79" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="80" spans="1:17">
+      <c r="A80" s="1">
+        <v>78</v>
+      </c>
+      <c r="B80" t="s">
+        <v>94</v>
+      </c>
+      <c r="C80">
+        <v>1</v>
+      </c>
+      <c r="D80" t="s">
+        <v>131</v>
+      </c>
+      <c r="E80" s="2">
+        <v>45137.4056283511</v>
+      </c>
+      <c r="P80" t="s">
+        <v>144</v>
+      </c>
+      <c r="Q80" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="81" spans="1:17">
+      <c r="A81" s="1">
+        <v>79</v>
+      </c>
+      <c r="B81" t="s">
+        <v>95</v>
+      </c>
+      <c r="C81">
+        <v>1</v>
+      </c>
+      <c r="D81" t="s">
+        <v>131</v>
+      </c>
+      <c r="E81" s="2">
+        <v>45137.40577930353</v>
+      </c>
+      <c r="P81" t="s">
+        <v>144</v>
+      </c>
+      <c r="Q81" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="82" spans="1:17">
+      <c r="A82" s="1">
+        <v>80</v>
+      </c>
+      <c r="B82" t="s">
+        <v>96</v>
+      </c>
+      <c r="C82">
+        <v>1</v>
+      </c>
+      <c r="D82" t="s">
+        <v>130</v>
+      </c>
+      <c r="E82" s="2">
+        <v>45137.41432293622</v>
+      </c>
+      <c r="P82" t="s">
+        <v>144</v>
+      </c>
+      <c r="Q82" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="83" spans="1:17">
+      <c r="A83" s="1">
+        <v>81</v>
+      </c>
+      <c r="B83" t="s">
+        <v>97</v>
+      </c>
+      <c r="C83">
+        <v>1</v>
+      </c>
+      <c r="D83" t="s">
+        <v>132</v>
+      </c>
+      <c r="E83" s="2">
+        <v>45137.4143230812</v>
+      </c>
+      <c r="P83" t="s">
+        <v>145</v>
+      </c>
+      <c r="Q83" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="84" spans="1:17">
+      <c r="A84" s="1">
+        <v>82</v>
+      </c>
+      <c r="B84" t="s">
+        <v>98</v>
+      </c>
+      <c r="C84">
+        <v>1</v>
+      </c>
+      <c r="D84" t="s">
+        <v>130</v>
+      </c>
+      <c r="E84" s="2">
+        <v>45137.4143984379</v>
+      </c>
+      <c r="P84" t="s">
+        <v>144</v>
+      </c>
+      <c r="Q84" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="85" spans="1:17">
+      <c r="A85" s="1">
+        <v>83</v>
+      </c>
+      <c r="B85" t="s">
+        <v>99</v>
+      </c>
+      <c r="C85">
+        <v>1</v>
+      </c>
+      <c r="D85" t="s">
+        <v>129</v>
+      </c>
+      <c r="E85" s="2">
+        <v>45137.41971360261</v>
+      </c>
+      <c r="P85" t="s">
+        <v>143</v>
+      </c>
+      <c r="Q85" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="86" spans="1:17">
+      <c r="A86" s="1">
+        <v>84</v>
+      </c>
+      <c r="B86" t="s">
+        <v>100</v>
+      </c>
+      <c r="C86">
+        <v>1</v>
+      </c>
+      <c r="D86" t="s">
+        <v>129</v>
+      </c>
+      <c r="E86" s="2">
+        <v>45137.41979940942</v>
+      </c>
+      <c r="P86" t="s">
+        <v>143</v>
+      </c>
+      <c r="Q86" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="87" spans="1:17">
+      <c r="A87" s="1">
+        <v>85</v>
+      </c>
+      <c r="B87" t="s">
+        <v>101</v>
+      </c>
+      <c r="C87">
+        <v>1</v>
+      </c>
+      <c r="D87" t="s">
+        <v>132</v>
+      </c>
+      <c r="E87" s="2">
+        <v>45137.41979955802</v>
+      </c>
+      <c r="P87" t="s">
+        <v>145</v>
+      </c>
+      <c r="Q87" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="88" spans="1:17">
+      <c r="A88" s="1">
+        <v>86</v>
+      </c>
+      <c r="B88" t="s">
+        <v>102</v>
+      </c>
+      <c r="C88">
+        <v>1</v>
+      </c>
+      <c r="D88" t="s">
+        <v>133</v>
+      </c>
+      <c r="E88" s="2">
+        <v>45137.41979971286</v>
+      </c>
+      <c r="O88" t="s">
+        <v>142</v>
+      </c>
+      <c r="P88" t="s">
+        <v>146</v>
+      </c>
+      <c r="Q88" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="89" spans="1:17">
+      <c r="A89" s="1">
+        <v>87</v>
+      </c>
+      <c r="B89" t="s">
+        <v>103</v>
+      </c>
+      <c r="C89">
+        <v>1</v>
+      </c>
+      <c r="D89" t="s">
+        <v>129</v>
+      </c>
+      <c r="E89" s="2">
+        <v>45137.41987869835</v>
+      </c>
+      <c r="P89" t="s">
+        <v>143</v>
+      </c>
+      <c r="Q89" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="90" spans="1:17">
+      <c r="A90" s="1">
+        <v>88</v>
+      </c>
+      <c r="B90" t="s">
+        <v>104</v>
+      </c>
+      <c r="C90">
+        <v>1</v>
+      </c>
+      <c r="D90" t="s">
+        <v>134</v>
+      </c>
+      <c r="E90" s="2">
+        <v>45137.41987890821</v>
+      </c>
+      <c r="O90" t="s">
+        <v>142</v>
+      </c>
+      <c r="P90" t="s">
+        <v>147</v>
+      </c>
+      <c r="Q90" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="91" spans="1:17">
+      <c r="A91" s="1">
+        <v>89</v>
+      </c>
+      <c r="B91" t="s">
+        <v>105</v>
+      </c>
+      <c r="C91">
+        <v>1</v>
+      </c>
+      <c r="D91" t="s">
+        <v>133</v>
+      </c>
+      <c r="E91" s="2">
+        <v>45137.4198791868</v>
+      </c>
+      <c r="O91" t="s">
+        <v>142</v>
+      </c>
+      <c r="P91" t="s">
+        <v>146</v>
+      </c>
+      <c r="Q91" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="92" spans="1:17">
+      <c r="A92" s="1">
+        <v>90</v>
+      </c>
+      <c r="B92" t="s">
+        <v>106</v>
+      </c>
+      <c r="C92">
+        <v>1</v>
+      </c>
+      <c r="D92" t="s">
+        <v>129</v>
+      </c>
+      <c r="E92" s="2">
+        <v>45137.41996190103</v>
+      </c>
+      <c r="P92" t="s">
+        <v>143</v>
+      </c>
+      <c r="Q92" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="93" spans="1:17">
+      <c r="A93" s="1">
+        <v>91</v>
+      </c>
+      <c r="B93" t="s">
         <v>107</v>
       </c>
-      <c r="Q77" t="s">
+      <c r="C93">
+        <v>1</v>
+      </c>
+      <c r="D93" t="s">
+        <v>132</v>
+      </c>
+      <c r="E93" s="2">
+        <v>45137.41996205963</v>
+      </c>
+      <c r="O93" t="s">
+        <v>142</v>
+      </c>
+      <c r="P93" t="s">
+        <v>145</v>
+      </c>
+      <c r="Q93" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="94" spans="1:17">
+      <c r="A94" s="1">
+        <v>92</v>
+      </c>
+      <c r="B94" t="s">
+        <v>108</v>
+      </c>
+      <c r="C94">
+        <v>1</v>
+      </c>
+      <c r="D94" t="s">
+        <v>133</v>
+      </c>
+      <c r="E94" s="2">
+        <v>45137.41996223558</v>
+      </c>
+      <c r="O94" t="s">
+        <v>142</v>
+      </c>
+      <c r="P94" t="s">
+        <v>146</v>
+      </c>
+      <c r="Q94" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="95" spans="1:17">
+      <c r="A95" s="1">
+        <v>93</v>
+      </c>
+      <c r="B95" t="s">
+        <v>109</v>
+      </c>
+      <c r="C95">
+        <v>1</v>
+      </c>
+      <c r="D95" t="s">
+        <v>129</v>
+      </c>
+      <c r="E95" s="2">
+        <v>45137.4200431575</v>
+      </c>
+      <c r="P95" t="s">
+        <v>143</v>
+      </c>
+      <c r="Q95" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="96" spans="1:17">
+      <c r="A96" s="1">
+        <v>94</v>
+      </c>
+      <c r="B96" t="s">
+        <v>110</v>
+      </c>
+      <c r="C96">
+        <v>1</v>
+      </c>
+      <c r="D96" t="s">
+        <v>134</v>
+      </c>
+      <c r="E96" s="2">
+        <v>45137.42004337583</v>
+      </c>
+      <c r="P96" t="s">
+        <v>147</v>
+      </c>
+      <c r="Q96" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="97" spans="1:17">
+      <c r="A97" s="1">
+        <v>95</v>
+      </c>
+      <c r="B97" t="s">
+        <v>111</v>
+      </c>
+      <c r="C97">
+        <v>1</v>
+      </c>
+      <c r="D97" t="s">
+        <v>132</v>
+      </c>
+      <c r="E97" s="2">
+        <v>45137.4200435892</v>
+      </c>
+      <c r="O97" t="s">
+        <v>142</v>
+      </c>
+      <c r="P97" t="s">
+        <v>145</v>
+      </c>
+      <c r="Q97" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="98" spans="1:17">
+      <c r="A98" s="1">
+        <v>96</v>
+      </c>
+      <c r="B98" t="s">
         <v>112</v>
+      </c>
+      <c r="C98">
+        <v>1</v>
+      </c>
+      <c r="D98" t="s">
+        <v>135</v>
+      </c>
+      <c r="E98" s="2">
+        <v>45137.42004384429</v>
+      </c>
+      <c r="P98" t="s">
+        <v>146</v>
+      </c>
+      <c r="Q98" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="99" spans="1:17">
+      <c r="A99" s="1">
+        <v>97</v>
+      </c>
+      <c r="B99" t="s">
+        <v>113</v>
+      </c>
+      <c r="C99">
+        <v>1</v>
+      </c>
+      <c r="D99" t="s">
+        <v>129</v>
+      </c>
+      <c r="E99" s="2">
+        <v>45137.42012374883</v>
+      </c>
+      <c r="P99" t="s">
+        <v>143</v>
+      </c>
+      <c r="Q99" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="100" spans="1:17">
+      <c r="A100" s="1">
+        <v>98</v>
+      </c>
+      <c r="B100" t="s">
+        <v>114</v>
+      </c>
+      <c r="C100">
+        <v>1</v>
+      </c>
+      <c r="D100" t="s">
+        <v>134</v>
+      </c>
+      <c r="E100" s="2">
+        <v>45137.42012395155</v>
+      </c>
+      <c r="O100" t="s">
+        <v>142</v>
+      </c>
+      <c r="P100" t="s">
+        <v>147</v>
+      </c>
+      <c r="Q100" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="101" spans="1:17">
+      <c r="A101" s="1">
+        <v>99</v>
+      </c>
+      <c r="B101" t="s">
+        <v>115</v>
+      </c>
+      <c r="C101">
+        <v>1</v>
+      </c>
+      <c r="D101" t="s">
+        <v>132</v>
+      </c>
+      <c r="E101" s="2">
+        <v>45137.42012412901</v>
+      </c>
+      <c r="O101" t="s">
+        <v>142</v>
+      </c>
+      <c r="P101" t="s">
+        <v>145</v>
+      </c>
+      <c r="Q101" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="102" spans="1:17">
+      <c r="A102" s="1">
+        <v>100</v>
+      </c>
+      <c r="B102" t="s">
+        <v>116</v>
+      </c>
+      <c r="C102">
+        <v>1</v>
+      </c>
+      <c r="D102" t="s">
+        <v>133</v>
+      </c>
+      <c r="E102" s="2">
+        <v>45137.4201253572</v>
+      </c>
+      <c r="O102" t="s">
+        <v>142</v>
+      </c>
+      <c r="P102" t="s">
+        <v>146</v>
+      </c>
+      <c r="Q102" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="103" spans="1:17">
+      <c r="A103" s="1">
+        <v>101</v>
+      </c>
+      <c r="B103" t="s">
+        <v>117</v>
+      </c>
+      <c r="C103">
+        <v>1</v>
+      </c>
+      <c r="D103" t="s">
+        <v>129</v>
+      </c>
+      <c r="E103" s="2">
+        <v>45137.420207403</v>
+      </c>
+      <c r="P103" t="s">
+        <v>143</v>
+      </c>
+      <c r="Q103" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="104" spans="1:17">
+      <c r="A104" s="1">
+        <v>102</v>
+      </c>
+      <c r="B104" t="s">
+        <v>118</v>
+      </c>
+      <c r="C104">
+        <v>1</v>
+      </c>
+      <c r="D104" t="s">
+        <v>136</v>
+      </c>
+      <c r="E104" s="2">
+        <v>45137.42020758646</v>
+      </c>
+      <c r="P104" t="s">
+        <v>147</v>
+      </c>
+      <c r="Q104" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="105" spans="1:17">
+      <c r="A105" s="1">
+        <v>103</v>
+      </c>
+      <c r="B105" t="s">
+        <v>119</v>
+      </c>
+      <c r="C105">
+        <v>1</v>
+      </c>
+      <c r="D105" t="s">
+        <v>137</v>
+      </c>
+      <c r="E105" s="2">
+        <v>45137.42020775888</v>
+      </c>
+      <c r="O105" t="s">
+        <v>142</v>
+      </c>
+      <c r="P105" t="s">
+        <v>145</v>
+      </c>
+      <c r="Q105" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="106" spans="1:17">
+      <c r="A106" s="1">
+        <v>104</v>
+      </c>
+      <c r="B106" t="s">
+        <v>120</v>
+      </c>
+      <c r="C106">
+        <v>1</v>
+      </c>
+      <c r="D106" t="s">
+        <v>133</v>
+      </c>
+      <c r="E106" s="2">
+        <v>45137.42020794875</v>
+      </c>
+      <c r="O106" t="s">
+        <v>142</v>
+      </c>
+      <c r="P106" t="s">
+        <v>146</v>
+      </c>
+      <c r="Q106" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="107" spans="1:17">
+      <c r="A107" s="1">
+        <v>105</v>
+      </c>
+      <c r="B107" t="s">
+        <v>121</v>
+      </c>
+      <c r="C107">
+        <v>1</v>
+      </c>
+      <c r="D107" t="s">
+        <v>129</v>
+      </c>
+      <c r="E107" s="2">
+        <v>45137.42028782015</v>
+      </c>
+      <c r="P107" t="s">
+        <v>143</v>
+      </c>
+      <c r="Q107" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="108" spans="1:17">
+      <c r="A108" s="1">
+        <v>106</v>
+      </c>
+      <c r="B108" t="s">
+        <v>122</v>
+      </c>
+      <c r="C108">
+        <v>1</v>
+      </c>
+      <c r="D108" t="s">
+        <v>134</v>
+      </c>
+      <c r="E108" s="2">
+        <v>45137.4202880244</v>
+      </c>
+      <c r="P108" t="s">
+        <v>147</v>
+      </c>
+      <c r="Q108" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="109" spans="1:17">
+      <c r="A109" s="1">
+        <v>107</v>
+      </c>
+      <c r="B109" t="s">
+        <v>123</v>
+      </c>
+      <c r="C109">
+        <v>1</v>
+      </c>
+      <c r="D109" t="s">
+        <v>138</v>
+      </c>
+      <c r="E109" s="2">
+        <v>45137.42028820136</v>
+      </c>
+      <c r="P109" t="s">
+        <v>145</v>
+      </c>
+      <c r="Q109" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="110" spans="1:17">
+      <c r="A110" s="1">
+        <v>108</v>
+      </c>
+      <c r="B110" t="s">
+        <v>124</v>
+      </c>
+      <c r="C110">
+        <v>1</v>
+      </c>
+      <c r="D110" t="s">
+        <v>133</v>
+      </c>
+      <c r="E110" s="2">
+        <v>45137.42028837808</v>
+      </c>
+      <c r="O110" t="s">
+        <v>142</v>
+      </c>
+      <c r="P110" t="s">
+        <v>146</v>
+      </c>
+      <c r="Q110" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="111" spans="1:17">
+      <c r="A111" s="1">
+        <v>109</v>
+      </c>
+      <c r="B111" t="s">
+        <v>125</v>
+      </c>
+      <c r="C111">
+        <v>1</v>
+      </c>
+      <c r="D111" t="s">
+        <v>129</v>
+      </c>
+      <c r="E111" s="2">
+        <v>45137.42036624673</v>
+      </c>
+      <c r="P111" t="s">
+        <v>143</v>
+      </c>
+      <c r="Q111" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="112" spans="1:17">
+      <c r="A112" s="1">
+        <v>110</v>
+      </c>
+      <c r="B112" t="s">
+        <v>126</v>
+      </c>
+      <c r="C112">
+        <v>1</v>
+      </c>
+      <c r="D112" t="s">
+        <v>136</v>
+      </c>
+      <c r="E112" s="2">
+        <v>45137.42036642238</v>
+      </c>
+      <c r="P112" t="s">
+        <v>147</v>
+      </c>
+      <c r="Q112" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="113" spans="1:17">
+      <c r="A113" s="1">
+        <v>111</v>
+      </c>
+      <c r="B113" t="s">
+        <v>127</v>
+      </c>
+      <c r="C113">
+        <v>1</v>
+      </c>
+      <c r="D113" t="s">
+        <v>138</v>
+      </c>
+      <c r="E113" s="2">
+        <v>45137.42036667763</v>
+      </c>
+      <c r="P113" t="s">
+        <v>145</v>
+      </c>
+      <c r="Q113" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="114" spans="1:17">
+      <c r="A114" s="1">
+        <v>112</v>
+      </c>
+      <c r="B114" t="s">
+        <v>128</v>
+      </c>
+      <c r="C114">
+        <v>1</v>
+      </c>
+      <c r="D114" t="s">
+        <v>135</v>
+      </c>
+      <c r="E114" s="2">
+        <v>45137.42036685873</v>
+      </c>
+      <c r="P114" t="s">
+        <v>146</v>
+      </c>
+      <c r="Q114" t="s">
+        <v>149</v>
       </c>
     </row>
   </sheetData>

</xml_diff>